<commit_message>
refactor: remove legacy Concur mapping feature
Removes the independent Concur Expense Type Mapping subsystem that
the previous two commits made obsolete: the admin "Concurマッピング"
tab and its CRUD state/validation, the Excel generator/importer
support for the "07_Concurマッピング" sheet (removed from both
sample-company.xlsm, via raw-ZIP surgery that leaves VBA/shapes/
comments untouched, and the initial-setup Excel template), and
config_snapshot's concur.expenseTypeMappings block. No expense type
IDs are renamed or guessed as part of this change; sample-company's
77 and company-a's 3 expense type IDs are byte-for-byte unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/templates/initial-setup-template.xlsx
+++ b/excel/templates/initial-setup-template.xlsx
@@ -11,14 +11,13 @@
     <sheet sheetId="5" name="04_質問" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="05_選択肢" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="99_記入ガイド" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="07_Concurマッピング" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="462">
   <si>
     <t>Concur迷子防止Bot 初期設定テンプレート</t>
   </si>
@@ -1235,9 +1234,6 @@
     <t>05_選択肢 … 選択肢・分岐・最終結果（旧仕様の06_判定ルールはこのシートに統合され廃止されました）</t>
   </si>
   <si>
-    <t>07_Concurマッピング … Concur Expense Type mapping一覧（任意。Concur連携を使わない場合はシートごと省略できます）</t>
-  </si>
-  <si>
     <t>99_記入ガイド … このシート</t>
   </si>
   <si>
@@ -1373,27 +1369,6 @@
     <t>片方が「次の質問」でもう片方が「結果」の場合はエラーになります。必ずどちらかに統一してください。</t>
   </si>
   <si>
-    <t>■ 07_Concurマッピング（任意シート。Concur連携を使わない場合はシートごと省略できます）</t>
-  </si>
-  <si>
-    <t>会社ID：シートを使う場合は必須。01_基本設定の会社IDと同じ値を入力してください。</t>
-  </si>
-  <si>
-    <t>ポリシーID：シートを使う場合は必須。02_ポリシーに存在するIDを入力してください。</t>
-  </si>
-  <si>
-    <t>経費タイプID：シートを使う場合は必須。03_経費タイプに存在するIDを入力してください。</t>
-  </si>
-  <si>
-    <t>Concur Expense Type Code：シートを使う場合は必須。Concur側で確認できた値をそのまま入力してください</t>
-  </si>
-  <si>
-    <t xml:space="preserve">　（このガイドに記載の値はあくまで説明用の例であり、実在するConcurのコードではありません）。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">　同じ会社ID・ポリシーID・経費タイプIDの組み合わせを複数の行に記入することはできません。</t>
-  </si>
-  <si>
     <t>■ 使用有無=N の経費タイプ・ポリシーについて</t>
   </si>
   <si>
@@ -1424,16 +1399,10 @@
     <t xml:space="preserve">　・05_選択肢の質問フロー・分岐の設計そのもの（会社の実務プロセスに依存するため）</t>
   </si>
   <si>
-    <t xml:space="preserve">　・07_Concurマッピングの内容全体（Concur側から正式に確認できた値のみを使用し、推測で埋めない）</t>
-  </si>
-  <si>
     <t>空欄にした項目は、インポート時の確認画面で警告として表示されるため、人間が後からレビューできます。</t>
   </si>
   <si>
     <t>断定して埋めてしまうと、誤った経費タイプが案内される等、実害につながる可能性があります。</t>
-  </si>
-  <si>
-    <t>Concur Expense Type Code</t>
   </si>
 </sst>
 </file>
@@ -5826,7 +5795,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A98"/>
+  <dimension ref="A1:A88"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -5887,13 +5856,13 @@
         <v>405</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="21" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="22" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>407</v>
       </c>
     </row>
@@ -5902,13 +5871,13 @@
         <v>408</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="26" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="27" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>410</v>
       </c>
     </row>
@@ -5922,13 +5891,13 @@
         <v>412</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="31" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="32" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>414</v>
       </c>
     </row>
@@ -5957,13 +5926,13 @@
         <v>419</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="39" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="40" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>421</v>
       </c>
     </row>
@@ -5997,13 +5966,13 @@
         <v>427</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="48" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="49" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="3" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>429</v>
       </c>
     </row>
@@ -6044,12 +6013,12 @@
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>437</v>
+        <v>225</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>225</v>
+        <v>437</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
@@ -6059,12 +6028,12 @@
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>439</v>
+        <v>225</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>225</v>
+        <v>439</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
@@ -6072,13 +6041,13 @@
         <v>440</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="64" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="65" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="3" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>442</v>
       </c>
     </row>
@@ -6094,12 +6063,12 @@
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>445</v>
+        <v>225</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>225</v>
+        <v>445</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
@@ -6114,12 +6083,12 @@
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>448</v>
+        <v>225</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>225</v>
+        <v>448</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
@@ -6127,8 +6096,8 @@
         <v>449</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="76" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
         <v>450</v>
       </c>
     </row>
@@ -6147,33 +6116,28 @@
         <v>453</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    <row r="81" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="3" t="s">
         <v>454</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="3" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>458</v>
       </c>
     </row>
@@ -6190,85 +6154,10 @@
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>461</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="3" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>470</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>471</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: rename Excel column "経費タイプID" to "経費タイプコード"
Aligns the initial-setup Excel spec's user-facing label with the value
it actually holds (Concur's own Expense Type / EXP_KEY code, e.g.
"01063", "CSHRN") and fixes the import mismatch against completed
templates that already used "経費タイプコード". Internal keys
(expenseTypes[].id, flow candidate expenseTypeId) and the Concur Quick
Expense API's expenseTypeId field are unchanged. No backward
compatibility for the old header, per this importer's existing
latest-version-only policy.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/templates/initial-setup-template.xlsx
+++ b/excel/templates/initial-setup-template.xlsx
@@ -73,7 +73,7 @@
     <t>出張経費</t>
   </si>
   <si>
-    <t>経費タイプID</t>
+    <t>経費タイプコード</t>
   </si>
   <si>
     <t>経費タイプ名</t>
@@ -1261,7 +1261,7 @@
     <t>■ 03_経費タイプ</t>
   </si>
   <si>
-    <t>経費タイプID：必須。Concur側の経費タイプコードをそのまま使うことを強く推奨します（一意）。</t>
+    <t>経費タイプコード：必須。Concur側の経費タイプコードをそのまま使うことを強く推奨します（一意）。</t>
   </si>
   <si>
     <t>ポリシーID：必須。02_ポリシーに存在するIDを入力してください。</t>
@@ -1321,7 +1321,7 @@
     <t>次に質問する質問キー：次のアクションが「次の質問」の場合のみ必須。04_質問の質問キーを入力してください。</t>
   </si>
   <si>
-    <t>経費タイプID：次のアクションが「結果」の場合のみ必須。03_経費タイプの経費タイプIDを入力してください。</t>
+    <t>経費タイプコード：次のアクションが「結果」の場合のみ必須。03_経費タイプの経費タイプコードを入力してください。</t>
   </si>
   <si>
     <t>案内メッセージ：次のアクションが「結果」の場合のみ必須。ユーザーへの案内文です。</t>
@@ -1339,13 +1339,13 @@
     <t>【結果の設定例】</t>
   </si>
   <si>
-    <t>質問キー=q02, ボタンに表示する文字=タクシー, 次のアクション=結果, 経費タイプID=taxi, 案内メッセージ=「タクシー」を選択してください。</t>
+    <t>質問キー=q02, ボタンに表示する文字=タクシー, 次のアクション=結果, 経費タイプコード=taxi, 案内メッセージ=「タクシー」を選択してください。</t>
   </si>
   <si>
     <t>■ 複数候補（1つの選択肢に対して経費タイプの候補を複数表示したい場合）</t>
   </si>
   <si>
-    <t>同じ「質問キー」と同じ「ボタンに表示する文字」の行を複数記述し、経費タイプIDだけを変えてください。</t>
+    <t>同じ「質問キー」と同じ「ボタンに表示する文字」の行を複数記述し、経費タイプコードだけを変えてください。</t>
   </si>
   <si>
     <t>この2行は「同一の選択肢の、異なる候補」として扱われ、ユーザー画面では「候補となる経費タイプ」として複数表示されます。</t>
@@ -1354,7 +1354,7 @@
     <t>以下は例です（このガイド上の例であり、実際のシートには含まれていません）。</t>
   </si>
   <si>
-    <t>質問キー   | ボタンに表示する文字 | 次のアクション | 経費タイプID | 案内メッセージ</t>
+    <t>質問キー   | ボタンに表示する文字 | 次のアクション | 経費タイプコード | 案内メッセージ</t>
   </si>
   <si>
     <t>q99_sample | 郵送費               | 結果            | postage       | 「郵送費」を選択してください。</t>
@@ -1375,10 +1375,10 @@
     <t>使用有無をNにしても、経費タイプ／ポリシー自体はマスタとして残りますが、Botの案内では使用されません。</t>
   </si>
   <si>
-    <t>05_選択肢の経費タイプIDから、使用有無=Nの経費タイプを参照すること自体は禁止していません（Errorにはなりません）が、</t>
-  </si>
-  <si>
-    <t>実際にはユーザーへ案内されなくなるため、意図しない場合は使用有無をYに戻すか、参照を別の経費タイプIDに変更してください。</t>
+    <t>05_選択肢の経費タイプコードから、使用有無=Nの経費タイプを参照すること自体は禁止していません（Errorにはなりません）が、</t>
+  </si>
+  <si>
+    <t>実際にはユーザーへ案内されなくなるため、意図しない場合は使用有無をYに戻すか、参照を別の経費タイプコードに変更してください。</t>
   </si>
   <si>
     <t>■ 【AI向け】ChatGPT等でこのテンプレートを埋める場合の注意</t>

</xml_diff>